<commit_message>
🤖 [Robot Incassi] Sincronizzazione locali_non_incassati.xlsx
</commit_message>
<xml_diff>
--- a/locali_non_incassati.xlsx
+++ b/locali_non_incassati.xlsx
@@ -11138,16 +11138,12 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="E195" t="inlineStr">
-        <is>
-          <t>SAVERIO WG BIANCO</t>
-        </is>
-      </c>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr"/>
       <c r="F195" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G195" t="n">
         <v>0</v>
@@ -11158,10 +11154,10 @@
         </is>
       </c>
       <c r="I195" t="n">
-        <v>4154</v>
+        <v>-256</v>
       </c>
       <c r="J195" t="n">
-        <v>1076</v>
+        <v>0</v>
       </c>
       <c r="K195" t="n">
         <v>0</v>
@@ -11173,7 +11169,7 @@
         <v>0</v>
       </c>
       <c r="N195" t="n">
-        <v>228.47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="196">

</xml_diff>